<commit_message>
fear: refactor code task send token
</commit_message>
<xml_diff>
--- a/aspnet-core/src/HRMv2.Web.Host/wwwroot/template/Export-MezonToken.xlsx
+++ b/aspnet-core/src/HRMv2.Web.Host/wwwroot/template/Export-MezonToken.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\c-sharp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4E85D723-E2A9-4ACA-A607-E03CF85A49A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A755375A-6196-47C7-AD0D-785DF3158004}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>#</t>
   </si>
@@ -47,12 +47,27 @@
   <si>
     <t>Mezon Token</t>
   </si>
+  <si>
+    <t>Note</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Sent At</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <numFmts count="4">
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
+    <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="166" formatCode="[$-1010409]d/m/yyyy\ h:mm\ AM/PM;@"/>
+  </numFmts>
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -83,6 +98,12 @@
       <color rgb="FFFF0000"/>
       <name val="Times New Roman"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -101,10 +122,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -115,8 +137,22 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -330,27 +366,37 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D1000"/>
+  <dimension ref="A1:G1000"/>
   <sheetFormatPr defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.109375" customWidth="1"/>
     <col min="2" max="2" width="65.6640625" customWidth="1"/>
-    <col min="3" max="3" width="30.6640625" customWidth="1"/>
+    <col min="3" max="3" width="30.6640625" style="6" customWidth="1"/>
     <col min="4" max="4" width="29.88671875" customWidth="1"/>
-    <col min="5" max="6" width="14.44140625" customWidth="1"/>
+    <col min="5" max="5" width="25.5546875" style="5" customWidth="1"/>
+    <col min="6" max="6" width="27.21875" style="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="48" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="48" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3"/>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="3"/>
     </row>
     <row r="21" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="22" ht="15.75" customHeight="1" x14ac:dyDescent="0.3"/>

</xml_diff>